<commit_message>
Build 2 local membership checkout and tracker progress
</commit_message>
<xml_diff>
--- a/outputs/01a0c842-4deb-7473-8541-dd8cd69d6272/VidCircle_Requirements_Tracker.xlsx
+++ b/outputs/01a0c842-4deb-7473-8541-dd8cd69d6272/VidCircle_Requirements_Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2d7ab51fe1df4374"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R9deb44b404f34655"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R135901905ece4ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Ra7224acea19949a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -145,7 +145,7 @@
         <x:color rgb="FF286747"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5ED"/>
         </x:patternFill>
       </x:fill>
@@ -156,7 +156,7 @@
         <x:color rgb="FF88611B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3DA"/>
         </x:patternFill>
       </x:fill>
@@ -166,7 +166,7 @@
         <x:color rgb="FF5B6680"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF2F7"/>
         </x:patternFill>
       </x:fill>
@@ -177,7 +177,7 @@
         <x:color rgb="FF286747"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5ED"/>
         </x:patternFill>
       </x:fill>
@@ -188,7 +188,7 @@
         <x:color rgb="FF88611B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3DA"/>
         </x:patternFill>
       </x:fill>
@@ -198,7 +198,7 @@
         <x:color rgb="FF5B6680"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF2F7"/>
         </x:patternFill>
       </x:fill>
@@ -506,7 +506,7 @@
         <x:v>Build 1</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Accounts, channels, dashboard, upload and native playback work locally; user review is next.</x:v>
+        <x:v>Accounts, channels, dashboard, upload and native playback work locally; Build 1 is complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="50" customHeight="1">
@@ -650,25 +650,25 @@
       </x:c>
       <x:c r="B11" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A11,'Requirements'!$D$6:$D$95,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C11" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A11,'Requirements'!$D$6:$D$95,"In progress")</x:f>
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D11" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A11,'Requirements'!$D$6:$D$95,"Planned")</x:f>
-        <x:v>15</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
         <x:f>IF(D11=0,IF(C11=0,"Completed","In progress"),IF(B11+C11&gt;0,"In progress","Planned"))</x:f>
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>No plan or checkout flow yet; local simulated checkout comes before Razorpay Test.</x:v>
+        <x:v>Plan comparison, signed test checkout and order history work locally; receipts, plan changes and access rules remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2257,12 +2257,14 @@
         <x:v>Define Free, Bronze, Silver and Gold plans with increasing access</x:v>
       </x:c>
       <x:c r="D81" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E81" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F81" s="9" t="str"/>
+      <x:c r="F81" s="9" t="str">
+        <x:v>One server-owned plan catalogue exists; access rules are not enforced yet.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="44" customHeight="1">
       <x:c r="A82" s="10" t="str">
@@ -2275,12 +2277,14 @@
         <x:v>Limit Free premium videos, features, quality, watch time and downloads</x:v>
       </x:c>
       <x:c r="D82" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E82" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F82" s="9" t="str"/>
+      <x:c r="F82" s="9" t="str">
+        <x:v>Free limits are defined in the catalogue, not enforced yet.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="44" customHeight="1">
       <x:c r="A83" s="10" t="str">
@@ -2293,13 +2297,13 @@
         <x:v>Add paid benefits: access, quality, offline, priority, speed, courses, no ads and usage</x:v>
       </x:c>
       <x:c r="D83" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E83" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F83" s="9" t="str">
-        <x:v>Faster streaming can only be represented locally, not guaranteed.</x:v>
+        <x:v>Paid benefits are defined for comparison; enforcement is pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="44" customHeight="1">
@@ -2313,12 +2317,14 @@
         <x:v>Set pricing and monthly, quarterly and yearly validity for each plan</x:v>
       </x:c>
       <x:c r="D84" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E84" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F84" s="9" t="str"/>
+      <x:c r="F84" s="9" t="str">
+        <x:v>Illustrative INR prices and 30/90/365-day terms are defined in one API catalogue.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="44" customHeight="1">
       <x:c r="A85" s="10" t="str">
@@ -2331,12 +2337,14 @@
         <x:v>Show a feature comparison, renewal policy and upgrade eligibility</x:v>
       </x:c>
       <x:c r="D85" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E85" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F85" s="9" t="str"/>
+      <x:c r="F85" s="9" t="str">
+        <x:v>Comparison and renewal policy are shown; upgrade eligibility is pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="44" customHeight="1">
       <x:c r="A86" s="10" t="str">
@@ -2349,13 +2357,13 @@
         <x:v>Show status, remaining validity, next renewal, billing history and benefits</x:v>
       </x:c>
       <x:c r="D86" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E86" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F86" s="9" t="str">
-        <x:v>Dedicated subscription dashboard.</x:v>
+        <x:v>Current plan, expiry and local test-order history are shown; benefits and renewal are pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="44" customHeight="1">
@@ -2369,12 +2377,14 @@
         <x:v>Let users compare plans before purchase</x:v>
       </x:c>
       <x:c r="D87" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E87" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F87" s="9" t="str"/>
+      <x:c r="F87" s="9" t="str">
+        <x:v>Signed-in users can compare all four plans and billing terms locally.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="44" customHeight="1">
       <x:c r="A88" s="10" t="str">
@@ -2425,12 +2435,14 @@
         <x:v>Handle success, failure, cancellation, duplicates and network interruption</x:v>
       </x:c>
       <x:c r="D90" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E90" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F90" s="9" t="str"/>
+      <x:c r="F90" s="9" t="str">
+        <x:v>Local success, failure, cancellation and duplicate results work; broader interruption handling remains.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="44" customHeight="1">
       <x:c r="A91" s="10" t="str">
@@ -2443,13 +2455,13 @@
         <x:v>Verify payment before activating or changing a subscription</x:v>
       </x:c>
       <x:c r="D91" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E91" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F91" s="9" t="str">
-        <x:v>A failed or interrupted payment must not activate benefits.</x:v>
+        <x:v>A signed local result is verified before activation; subscription-change flows remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="44" customHeight="1">
@@ -2463,12 +2475,14 @@
         <x:v>Store payment/order/invoice IDs, amount, currency, status, start/expiry and renewal</x:v>
       </x:c>
       <x:c r="D92" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E92" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F92" s="9" t="str"/>
+      <x:c r="F92" s="9" t="str">
+        <x:v>Local order and test-payment references, amount, currency, status and term are stored; renewal is pending.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="44" customHeight="1">
       <x:c r="A93" s="10" t="str">
@@ -2501,12 +2515,14 @@
         <x:v>Downgrade expired plans to Free while retaining user data and watch history</x:v>
       </x:c>
       <x:c r="D94" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E94" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F94" s="9" t="str"/>
+      <x:c r="F94" s="9" t="str">
+        <x:v>An expired paid record reads as Free without changing account or history; full expiry workflow remains.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="44" customHeight="1">
       <x:c r="A95" s="10" t="str">
@@ -2541,7 +2557,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re991cf89d19a4360"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R157f1eef25e846cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete local Build 2 access and Build 3 player
</commit_message>
<xml_diff>
--- a/outputs/01a0c842-4deb-7473-8541-dd8cd69d6272/VidCircle_Requirements_Tracker.xlsx
+++ b/outputs/01a0c842-4deb-7473-8541-dd8cd69d6272/VidCircle_Requirements_Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R135901905ece4ab4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Ra7224acea19949a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf4352249cb2e4613"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Re9f22e9c7a774b3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
         <x:v>Build 1</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Accounts, channels, dashboard, upload and native playback work locally; Build 1 is complete.</x:v>
+        <x:v>Build 1 completed accounts, channels, dashboard, upload and basic playback. The player was upgraded in Phase 3A.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="50" customHeight="1">
@@ -596,7 +596,7 @@
       </x:c>
       <x:c r="B9" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A9,'Requirements'!$D$6:$D$95,"Completed")</x:f>
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C9" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A9,'Requirements'!$D$6:$D$95,"In progress")</x:f>
@@ -604,7 +604,7 @@
       </x:c>
       <x:c r="D9" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A9,'Requirements'!$D$6:$D$95,"Planned")</x:f>
-        <x:v>14</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
         <x:f>IF(D9=0,IF(C9=0,"Completed","In progress"),IF(B9+C9&gt;0,"In progress","Planned"))</x:f>
@@ -614,7 +614,7 @@
         <x:v>Build 3</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>Uploaded MP4s play with browser controls; the requested custom player is not built.</x:v>
+        <x:v>Build 3 works locally: custom controls, saved progress, plan-capped quality, captions, timeline frames and next-video flow. Full-screen and PiP still need a supporting-browser check.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="50" customHeight="1">
@@ -650,15 +650,15 @@
       </x:c>
       <x:c r="B11" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A11,'Requirements'!$D$6:$D$95,"Completed")</x:f>
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C11" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A11,'Requirements'!$D$6:$D$95,"In progress")</x:f>
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D11" s="14" t="n">
         <x:f>COUNTIFS('Requirements'!$B$6:$B$95,$A11,'Requirements'!$D$6:$D$95,"Planned")</x:f>
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
         <x:f>IF(D11=0,IF(C11=0,"Completed","In progress"),IF(B11+C11&gt;0,"In progress","Planned"))</x:f>
@@ -668,7 +668,7 @@
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>Plan comparison, signed test checkout and order history work locally; receipts, plan changes and access rules remain.</x:v>
+        <x:v>Build 2 local prototype complete: checkout, plan gates, per-rendition quality caps, daily clip allowance, early access, ad placeholder and history. Original external/later benefits remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -949,7 +949,7 @@
         <x:v>Build 1</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>Browser playback and refresh were checked. Uses native controls.</x:v>
+        <x:v>Basic native MP4 playback was checked in Build 1; Build 3A now uses custom controls.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
@@ -1793,13 +1793,13 @@
         <x:v>Build a fully custom HTML5 player instead of browser-default controls</x:v>
       </x:c>
       <x:c r="D56" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E56" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
       <x:c r="F56" s="9" t="str">
-        <x:v>Basic native MP4 playback works; custom controls remain.</x:v>
+        <x:v>Custom HTML5 controls replace the browser controls on the watch page.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="44" customHeight="1">
@@ -1813,12 +1813,14 @@
         <x:v>Add custom play/pause, draggable volume and mute/unmute controls</x:v>
       </x:c>
       <x:c r="D57" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E57" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F57" s="9" t="str"/>
+      <x:c r="F57" s="9" t="str">
+        <x:v>Play/pause, draggable volume and mute/unmute work locally.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="44" customHeight="1">
       <x:c r="A58" s="10" t="str">
@@ -1831,12 +1833,14 @@
         <x:v>Offer 0.5x, 1x, 1.25x, 1.5x and 2x playback speeds</x:v>
       </x:c>
       <x:c r="D58" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E58" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F58" s="9" t="str"/>
+      <x:c r="F58" s="9" t="str">
+        <x:v>0.5x, 1x, 1.25x, 1.5x and 2x speeds work locally.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="44" customHeight="1">
       <x:c r="A59" s="10" t="str">
@@ -1849,12 +1853,14 @@
         <x:v>Seek backward/forward by 10 seconds and support larger skips</x:v>
       </x:c>
       <x:c r="D59" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E59" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F59" s="9" t="str"/>
+      <x:c r="F59" s="9" t="str">
+        <x:v>10-second buttons and arrows, plus 30-second Shift+arrow skips, work locally.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="44" customHeight="1">
       <x:c r="A60" s="10" t="str">
@@ -1867,12 +1873,14 @@
         <x:v>Support theatre mode, full-screen mode and Picture-in-Picture</x:v>
       </x:c>
       <x:c r="D60" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E60" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F60" s="9" t="str"/>
+      <x:c r="F60" s="9" t="str">
+        <x:v>Theatre mode works. Full-screen and PiP controls are implemented but need a normal-browser check.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="44" customHeight="1">
       <x:c r="A61" s="10" t="str">
@@ -1885,12 +1893,14 @@
         <x:v>Toggle subtitles or captions when available</x:v>
       </x:c>
       <x:c r="D61" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E61" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F61" s="9" t="str"/>
+      <x:c r="F61" s="9" t="str">
+        <x:v>Optional uploaded WebVTT captions load privately; the player button and C shortcut turn them on or off.</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="44" customHeight="1">
       <x:c r="A62" s="10" t="str">
@@ -1903,12 +1913,14 @@
         <x:v>Show current, total and remaining time</x:v>
       </x:c>
       <x:c r="D62" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E62" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F62" s="9" t="str"/>
+      <x:c r="F62" s="9" t="str">
+        <x:v>Current, total and remaining time are shown.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="44" customHeight="1">
       <x:c r="A63" s="10" t="str">
@@ -1921,12 +1933,14 @@
         <x:v>Show buffering, playback progress and loading indicators</x:v>
       </x:c>
       <x:c r="D63" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E63" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F63" s="9" t="str"/>
+      <x:c r="F63" s="9" t="str">
+        <x:v>Buffered and played portions, loading state and seek progress are shown.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="44" customHeight="1">
       <x:c r="A64" s="10" t="str">
@@ -1939,13 +1953,13 @@
         <x:v>Show video quality information and allow quality selection</x:v>
       </x:c>
       <x:c r="D64" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E64" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
       <x:c r="F64" s="9" t="str">
-        <x:v>Prepare local variants; plan checks come in Build 2.</x:v>
+        <x:v>New uploads create lower-resolution MP4s. The player lists qualities and the API enforces the active-plan cap on direct requests.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="44" customHeight="1">
@@ -1959,12 +1973,14 @@
         <x:v>Autoplay the next video after a countdown, with a cancel option</x:v>
       </x:c>
       <x:c r="D65" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E65" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F65" s="9" t="str"/>
+      <x:c r="F65" s="9" t="str">
+        <x:v>A five-second countdown offers the next watchable video, with Play now and Cancel; both paths were checked locally.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="44" customHeight="1">
       <x:c r="A66" s="10" t="str">
@@ -1977,12 +1993,14 @@
         <x:v>Save watch position periodically and resume from the last position</x:v>
       </x:c>
       <x:c r="D66" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E66" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F66" s="9" t="str"/>
+      <x:c r="F66" s="9" t="str">
+        <x:v>Position saves during playback and on pause, seek, end or exit. An unfinished video resumes across sessions.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="44" customHeight="1">
       <x:c r="A67" s="10" t="str">
@@ -1995,12 +2013,14 @@
         <x:v>Mark completion at a configurable watched percentage</x:v>
       </x:c>
       <x:c r="D67" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E67" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F67" s="9" t="str"/>
+      <x:c r="F67" s="9" t="str">
+        <x:v>The local threshold defaults to 90% of accumulated playback time. Skips do not count; replayed time can count again.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="44" customHeight="1">
       <x:c r="A68" s="10" t="str">
@@ -2013,12 +2033,14 @@
         <x:v>Prevent multiple videos from playing simultaneously across open app tabs</x:v>
       </x:c>
       <x:c r="D68" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E68" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F68" s="9" t="str"/>
+      <x:c r="F68" s="9" t="str">
+        <x:v>Starting another VidCircle tab pauses the older player in the same browser profile.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="44" customHeight="1">
       <x:c r="A69" s="10" t="str">
@@ -2031,13 +2053,13 @@
         <x:v>Implement space, arrow, Shift-arrow, volume and dedicated desktop shortcuts</x:v>
       </x:c>
       <x:c r="D69" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E69" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
       <x:c r="F69" s="9" t="str">
-        <x:v>Includes mute, speed, PiP, theatre, captions, full-screen and next.</x:v>
+        <x:v>Playback, seek, volume, mute, speed, theatre, full-screen, PiP, captions, next-video and help shortcuts are implemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="44" customHeight="1">
@@ -2051,12 +2073,14 @@
         <x:v>Show frame previews on timeline hover and auto-hide/reveal controls on mouse activity</x:v>
       </x:c>
       <x:c r="D70" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E70" s="11" t="str">
         <x:v>Build 3</x:v>
       </x:c>
-      <x:c r="F70" s="9" t="str"/>
+      <x:c r="F70" s="9" t="str">
+        <x:v>Generated frames appear on timeline pointer movement; controls hide during playback and reappear on activity.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="44" customHeight="1">
       <x:c r="A71" s="10" t="str">
@@ -2257,13 +2281,13 @@
         <x:v>Define Free, Bronze, Silver and Gold plans with increasing access</x:v>
       </x:c>
       <x:c r="D81" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E81" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F81" s="9" t="str">
-        <x:v>One server-owned plan catalogue exists; access rules are not enforced yet.</x:v>
+        <x:v>Four plans, terms, tiered video access, source-resolution rules and daily allowances work locally.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="44" customHeight="1">
@@ -2283,7 +2307,7 @@
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F82" s="9" t="str">
-        <x:v>Free limits are defined in the catalogue, not enforced yet.</x:v>
+        <x:v>Free can watch 480p copies of new HD uploads; protected quality requests and the daily watch allowance work. Downloads remain Build 5.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="44" customHeight="1">
@@ -2303,7 +2327,7 @@
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F83" s="9" t="str">
-        <x:v>Paid benefits are defined for comparison; enforcement is pending.</x:v>
+        <x:v>Paid resolution tiers, access, Gold early access, usage, speed and ad-free placeholder work. Offline and courses remain later work.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="44" customHeight="1">
@@ -2337,13 +2361,13 @@
         <x:v>Show a feature comparison, renewal policy and upgrade eligibility</x:v>
       </x:c>
       <x:c r="D85" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E85" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F85" s="9" t="str">
-        <x:v>Comparison and renewal policy are shown; upgrade eligibility is pending.</x:v>
+        <x:v>Comparison, manual renewal policy and current-plan upgrade eligibility are shown locally.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="44" customHeight="1">
@@ -2357,13 +2381,13 @@
         <x:v>Show status, remaining validity, next renewal, billing history and benefits</x:v>
       </x:c>
       <x:c r="D86" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E86" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F86" s="9" t="str">
-        <x:v>Current plan, expiry and local test-order history are shown; benefits and renewal are pending.</x:v>
+        <x:v>Current plan, remaining days, expiry, scheduled change, order history and benefits are shown. Renewal is manual in the local prototype.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="44" customHeight="1">
@@ -2397,12 +2421,14 @@
         <x:v>Support upgrade, downgrade, renewal and cancellation</x:v>
       </x:c>
       <x:c r="D88" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E88" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
-      <x:c r="F88" s="9" t="str"/>
+      <x:c r="F88" s="9" t="str">
+        <x:v>Verified local orders can renew, upgrade or schedule a prepaid downgrade; cancellation ends access after paid terms.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="44" customHeight="1">
       <x:c r="A89" s="10" t="str">
@@ -2435,13 +2461,13 @@
         <x:v>Handle success, failure, cancellation, duplicates and network interruption</x:v>
       </x:c>
       <x:c r="D90" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E90" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F90" s="9" t="str">
-        <x:v>Local success, failure, cancellation and duplicate results work; broader interruption handling remains.</x:v>
+        <x:v>Success, failure, cancellation, duplicate results, stale orders and interrupted verification recovery pass local API tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="44" customHeight="1">
@@ -2455,13 +2481,13 @@
         <x:v>Verify payment before activating or changing a subscription</x:v>
       </x:c>
       <x:c r="D91" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E91" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F91" s="9" t="str">
-        <x:v>A signed local result is verified before activation; subscription-change flows remain.</x:v>
+        <x:v>A signed local result must be verified before purchase, renewal, upgrade or downgrade changes membership.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="44" customHeight="1">
@@ -2475,13 +2501,13 @@
         <x:v>Store payment/order/invoice IDs, amount, currency, status, start/expiry and renewal</x:v>
       </x:c>
       <x:c r="D92" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E92" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F92" s="9" t="str">
-        <x:v>Local order and test-payment references, amount, currency, status and term are stored; renewal is pending.</x:v>
+        <x:v>Local order, test-payment and receipt references, amount, currency, status and term dates are stored; renewals extend expiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="44" customHeight="1">
@@ -2495,13 +2521,13 @@
         <x:v>Enforce premium access on the server</x:v>
       </x:c>
       <x:c r="D93" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E93" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F93" s="9" t="str">
-        <x:v>Protected media access begins in Build 2.</x:v>
+        <x:v>Every authenticated media request checks the current plan, source resolution, early-access window and daily allowance; public upload URLs are closed.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="44" customHeight="1">
@@ -2515,13 +2541,13 @@
         <x:v>Downgrade expired plans to Free while retaining user data and watch history</x:v>
       </x:c>
       <x:c r="D94" s="8" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="E94" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F94" s="9" t="str">
-        <x:v>An expired paid record reads as Free without changing account or history; full expiry workflow remains.</x:v>
+        <x:v>Expired terms become Free; protected watch history remains visible and owner-only after expiry.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="44" customHeight="1">
@@ -2535,13 +2561,13 @@
         <x:v>Email invoice, receipt, plan, validity, transaction and support details</x:v>
       </x:c>
       <x:c r="D95" s="8" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E95" s="11" t="str">
         <x:v>Build 2</x:v>
       </x:c>
       <x:c r="F95" s="9" t="str">
-        <x:v>Start with Mailpit; real email delivery is later.</x:v>
+        <x:v>A local test receipt shows plan, validity, payment reference and support; Mailpit captures email. No tax invoice or real delivery.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2557,7 +2583,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R157f1eef25e846cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73da3cae5c2f4ad7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>